<commit_message>
Régénère les figures et tableaux de référence sur le banc corrigé
Exécution de run_all (graine 42) avec l'entraînement à arrêt anticipé,
le garde-fou de bout en bout et la continuité de la ligne à retards.

Les figures reflètent désormais un réseau à -21,2 dB en nominal et
non plus -18,8 dB. Le pic de -8 dB du bloc 16 de S2, décrit dans le
mémoire comme transitoire de crête, a disparu : il était l'artefact
des M premiers échantillons non prédistordus de chaque bloc. Les
courbes statique et adaptative se superposent désormais sur tous les
scénarios.

Les anciennes figures sont conservées dans
results/figures/archive_v1_5epoques/.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ANfZS1oHgEptxBRYH8Zhc7
</commit_message>
<xml_diff>
--- a/results/tables/summary_all_scenarios.xlsx
+++ b/results/tables/summary_all_scenarios.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4219" uniqueCount="2137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4462" uniqueCount="2260">
   <si>
     <t>Scenario</t>
   </si>
@@ -1480,6 +1480,375 @@
   </si>
   <si>
     <t>ACPR_dBc_before</t>
+  </si>
+  <si>
+    <t>ACPR_dBc_after</t>
+  </si>
+  <si>
+    <t>NumAdaptations</t>
+  </si>
+  <si>
+    <t>Runtime_s</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>Calibration nominale et référence de performance</t>
+  </si>
+  <si>
+    <t>Static MP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Static GMP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Offline NN-DPD with fixed weights</t>
+  </si>
+  <si>
+    <t>Online NN-DPD adaptation</t>
+  </si>
+  <si>
+    <t>Dérive thermique graduelle du PA</t>
+  </si>
+  <si>
+    <t>Static MP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Static GMP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Offline NN-DPD with fixed weights</t>
+  </si>
+  <si>
+    <t>Online NN-DPD adaptation</t>
+  </si>
+  <si>
+    <t>Rupture brutale de puissance ou changement d IBO</t>
+  </si>
+  <si>
+    <t>Static MP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Static GMP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Offline NN-DPD with fixed weights</t>
+  </si>
+  <si>
+    <t>Online NN-DPD adaptation</t>
+  </si>
+  <si>
+    <t>Variation des effets mémoire du PA</t>
+  </si>
+  <si>
+    <t>Static MP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Static GMP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Offline NN-DPD with fixed weights</t>
+  </si>
+  <si>
+    <t>Online NN-DPD adaptation</t>
+  </si>
+  <si>
+    <t>Vieillissement lent du PA</t>
+  </si>
+  <si>
+    <t>Static MP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Static GMP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Offline NN-DPD with fixed weights</t>
+  </si>
+  <si>
+    <t>Online NN-DPD adaptation</t>
+  </si>
+  <si>
+    <t>Variation de charge, désadaptation ou effet VSWR</t>
+  </si>
+  <si>
+    <t>Static MP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Static GMP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Offline NN-DPD with fixed weights</t>
+  </si>
+  <si>
+    <t>Online NN-DPD adaptation</t>
+  </si>
+  <si>
+    <t>Dérive combinée thermique + puissance + mémoire + charge</t>
+  </si>
+  <si>
+    <t>Static MP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Static GMP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Offline NN-DPD with fixed weights</t>
+  </si>
+  <si>
+    <t>Online NN-DPD adaptation</t>
+  </si>
+  <si>
+    <t>Stress test 5G NR avec variation de bande, modulation et numérologie</t>
+  </si>
+  <si>
+    <t>Static MP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Static GMP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Offline NN-DPD with fixed weights</t>
+  </si>
+  <si>
+    <t>Online NN-DPD adaptation</t>
+  </si>
+  <si>
+    <t>Optimisation de la politique d adaptation par RL ou heuristique</t>
+  </si>
+  <si>
+    <t>Static MP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Static GMP-DPD baseline</t>
+  </si>
+  <si>
+    <t>Offline NN-DPD with fixed weights</t>
+  </si>
+  <si>
+    <t>Online NN-DPD adaptation</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>S0</t>
+  </si>
+  <si>
+    <t>S1</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t>S4</t>
+  </si>
+  <si>
+    <t>S5</t>
+  </si>
+  <si>
+    <t>S6</t>
+  </si>
+  <si>
+    <t>S7</t>
+  </si>
+  <si>
+    <t>S8</t>
+  </si>
+  <si>
+    <t>Waveform</t>
+  </si>
+  <si>
+    <t>OFDM-QAM</t>
+  </si>
+  <si>
+    <t>5GNR</t>
+  </si>
+  <si>
+    <t>OFDM-QAM</t>
+  </si>
+  <si>
+    <t>Modulation</t>
+  </si>
+  <si>
+    <t>64QAM</t>
+  </si>
+  <si>
+    <t>256QAM</t>
+  </si>
+  <si>
+    <t>64QAM</t>
+  </si>
+  <si>
+    <t>Bandwidth_MHz</t>
+  </si>
+  <si>
+    <t>IBO_dB</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>No_DPD</t>
+  </si>
+  <si>
+    <t>MP_DPD</t>
+  </si>
+  <si>
+    <t>GMP_DPD</t>
+  </si>
+  <si>
+    <t>NN_DPD_Static</t>
+  </si>
+  <si>
+    <t>NN_DPD_Adaptive</t>
+  </si>
+  <si>
+    <t>No_DPD</t>
+  </si>
+  <si>
+    <t>MP_DPD</t>
+  </si>
+  <si>
+    <t>GMP_DPD</t>
+  </si>
+  <si>
+    <t>NN_DPD_Static</t>
+  </si>
+  <si>
+    <t>NN_DPD_Adaptive</t>
+  </si>
+  <si>
+    <t>No_DPD</t>
+  </si>
+  <si>
+    <t>MP_DPD</t>
+  </si>
+  <si>
+    <t>GMP_DPD</t>
+  </si>
+  <si>
+    <t>NN_DPD_Static</t>
+  </si>
+  <si>
+    <t>NN_DPD_Adaptive</t>
+  </si>
+  <si>
+    <t>No_DPD</t>
+  </si>
+  <si>
+    <t>MP_DPD</t>
+  </si>
+  <si>
+    <t>GMP_DPD</t>
+  </si>
+  <si>
+    <t>NN_DPD_Static</t>
+  </si>
+  <si>
+    <t>NN_DPD_Adaptive</t>
+  </si>
+  <si>
+    <t>No_DPD</t>
+  </si>
+  <si>
+    <t>MP_DPD</t>
+  </si>
+  <si>
+    <t>GMP_DPD</t>
+  </si>
+  <si>
+    <t>NN_DPD_Static</t>
+  </si>
+  <si>
+    <t>NN_DPD_Adaptive</t>
+  </si>
+  <si>
+    <t>No_DPD</t>
+  </si>
+  <si>
+    <t>MP_DPD</t>
+  </si>
+  <si>
+    <t>GMP_DPD</t>
+  </si>
+  <si>
+    <t>NN_DPD_Static</t>
+  </si>
+  <si>
+    <t>NN_DPD_Adaptive</t>
+  </si>
+  <si>
+    <t>No_DPD</t>
+  </si>
+  <si>
+    <t>MP_DPD</t>
+  </si>
+  <si>
+    <t>GMP_DPD</t>
+  </si>
+  <si>
+    <t>NN_DPD_Static</t>
+  </si>
+  <si>
+    <t>NN_DPD_Adaptive</t>
+  </si>
+  <si>
+    <t>No_DPD</t>
+  </si>
+  <si>
+    <t>MP_DPD</t>
+  </si>
+  <si>
+    <t>GMP_DPD</t>
+  </si>
+  <si>
+    <t>NN_DPD_Static</t>
+  </si>
+  <si>
+    <t>NN_DPD_Adaptive</t>
+  </si>
+  <si>
+    <t>No_DPD</t>
+  </si>
+  <si>
+    <t>MP_DPD</t>
+  </si>
+  <si>
+    <t>GMP_DPD</t>
+  </si>
+  <si>
+    <t>NN_DPD_Static</t>
+  </si>
+  <si>
+    <t>RL_Adaptive_Policy</t>
+  </si>
+  <si>
+    <t>NMSE_dB_before</t>
+  </si>
+  <si>
+    <t>NMSE_dB_during</t>
+  </si>
+  <si>
+    <t>NMSE_dB_after</t>
+  </si>
+  <si>
+    <t>EVM_percent_before</t>
+  </si>
+  <si>
+    <t>EVM_percent_during</t>
+  </si>
+  <si>
+    <t>EVM_percent_after</t>
+  </si>
+  <si>
+    <t>ACPR_dBc_before</t>
+  </si>
+  <si>
+    <t>ACPR_dBc_during</t>
   </si>
   <si>
     <t>ACPR_dBc_after</t>
@@ -6494,69 +6863,69 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>2014</v>
+        <v>2137</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>2024</v>
+        <v>2147</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2028</v>
+        <v>2151</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>2032</v>
+        <v>2155</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>2033</v>
+        <v>2156</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>2034</v>
+        <v>2157</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>2080</v>
+        <v>2203</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>2081</v>
+        <v>2204</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>2082</v>
+        <v>2205</v>
       </c>
       <c r="J1" s="0" t="s">
-        <v>2083</v>
+        <v>2206</v>
       </c>
       <c r="K1" s="0" t="s">
-        <v>2084</v>
+        <v>2207</v>
       </c>
       <c r="L1" s="0" t="s">
-        <v>2085</v>
+        <v>2208</v>
       </c>
       <c r="M1" s="0" t="s">
-        <v>2086</v>
+        <v>2209</v>
       </c>
       <c r="N1" s="0" t="s">
-        <v>2087</v>
+        <v>2210</v>
       </c>
       <c r="O1" s="0" t="s">
-        <v>2088</v>
+        <v>2211</v>
       </c>
       <c r="P1" s="0" t="s">
-        <v>2089</v>
+        <v>2212</v>
       </c>
       <c r="Q1" s="0" t="s">
-        <v>2090</v>
+        <v>2213</v>
       </c>
       <c r="R1" s="0" t="s">
-        <v>2091</v>
+        <v>2214</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>2015</v>
+        <v>2138</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D2" s="0">
         <v>40</v>
@@ -6565,7 +6934,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>2035</v>
+        <v>2158</v>
       </c>
       <c r="G2" s="0">
         <v>-5.5798344850129187</v>
@@ -6598,21 +6967,21 @@
         <v>0</v>
       </c>
       <c r="Q2" s="0">
-        <v>3.424320356</v>
+        <v>3.6013117779999999</v>
       </c>
       <c r="R2" s="0" t="s">
-        <v>2092</v>
+        <v>2215</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>2015</v>
+        <v>2138</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D3" s="0">
         <v>40</v>
@@ -6621,7 +6990,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>2036</v>
+        <v>2159</v>
       </c>
       <c r="G3" s="0">
         <v>-21.213114059865443</v>
@@ -6654,21 +7023,21 @@
         <v>0</v>
       </c>
       <c r="Q3" s="0">
-        <v>3.5955898510000002</v>
+        <v>3.8526201100000002</v>
       </c>
       <c r="R3" s="0" t="s">
-        <v>2093</v>
+        <v>2216</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>2015</v>
+        <v>2138</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D4" s="0">
         <v>40</v>
@@ -6677,7 +7046,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>2037</v>
+        <v>2160</v>
       </c>
       <c r="G4" s="0">
         <v>-21.161779043338118</v>
@@ -6710,21 +7079,21 @@
         <v>0</v>
       </c>
       <c r="Q4" s="0">
-        <v>3.6493906319999998</v>
+        <v>3.900402009</v>
       </c>
       <c r="R4" s="0" t="s">
-        <v>2094</v>
+        <v>2217</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>2015</v>
+        <v>2138</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D5" s="0">
         <v>40</v>
@@ -6733,54 +7102,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>2038</v>
+        <v>2161</v>
       </c>
       <c r="G5" s="0">
-        <v>-18.962492219096983</v>
+        <v>-21.558838442819713</v>
       </c>
       <c r="H5" s="0">
-        <v>-18.646400126470638</v>
+        <v>-20.950172756393005</v>
       </c>
       <c r="I5" s="0">
-        <v>-18.821265968913078</v>
+        <v>-21.194738694946938</v>
       </c>
       <c r="J5" s="0">
-        <v>11.268740788174608</v>
+        <v>8.3571477023684224</v>
       </c>
       <c r="K5" s="0">
-        <v>11.68637972398515</v>
+        <v>8.9637835742135419</v>
       </c>
       <c r="L5" s="0">
-        <v>11.453459950351188</v>
+        <v>8.7149131865844307</v>
       </c>
       <c r="M5" s="0">
-        <v>-33.596101862491295</v>
+        <v>-32.818440655441961</v>
       </c>
       <c r="N5" s="0">
-        <v>-32.838245869513607</v>
+        <v>-32.345624521338088</v>
       </c>
       <c r="O5" s="0">
-        <v>-32.490893433807045</v>
+        <v>-32.258605692896559</v>
       </c>
       <c r="P5" s="0">
         <v>0</v>
       </c>
       <c r="Q5" s="0">
-        <v>23.206771288999999</v>
+        <v>292.305066275</v>
       </c>
       <c r="R5" s="0" t="s">
-        <v>2095</v>
+        <v>2218</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>2015</v>
+        <v>2138</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D6" s="0">
         <v>40</v>
@@ -6789,54 +7158,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>2039</v>
+        <v>2162</v>
       </c>
       <c r="G6" s="0">
-        <v>-18.870557836214445</v>
+        <v>-21.503893193431654</v>
       </c>
       <c r="H6" s="0">
-        <v>-18.532315660711106</v>
+        <v>-20.907851582816328</v>
       </c>
       <c r="I6" s="0">
-        <v>-18.446621179771423</v>
+        <v>-21.074503510416282</v>
       </c>
       <c r="J6" s="0">
-        <v>11.388646379185753</v>
+        <v>8.410180956356335</v>
       </c>
       <c r="K6" s="0">
-        <v>11.840886465348976</v>
+        <v>9.0075653342622743</v>
       </c>
       <c r="L6" s="0">
-        <v>11.958286137997511</v>
+        <v>8.8363889618891545</v>
       </c>
       <c r="M6" s="0">
-        <v>-33.453707844069712</v>
+        <v>-32.69765719837477</v>
       </c>
       <c r="N6" s="0">
-        <v>-32.693715041080125</v>
+        <v>-32.255410532863017</v>
       </c>
       <c r="O6" s="0">
-        <v>-32.241393790211916</v>
+        <v>-32.078769870429163</v>
       </c>
       <c r="P6" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="0">
-        <v>25.080844408000001</v>
+        <v>293.41545357199999</v>
       </c>
       <c r="R6" s="0" t="s">
-        <v>2096</v>
+        <v>2219</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>2016</v>
+        <v>2139</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D7" s="0">
         <v>40</v>
@@ -6845,7 +7214,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>2040</v>
+        <v>2163</v>
       </c>
       <c r="G7" s="0">
         <v>-5.0259485033135469</v>
@@ -6878,21 +7247,21 @@
         <v>0</v>
       </c>
       <c r="Q7" s="0">
-        <v>3.6481320789999998</v>
+        <v>3.2221986550000001</v>
       </c>
       <c r="R7" s="0" t="s">
-        <v>2097</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>2016</v>
+        <v>2139</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D8" s="0">
         <v>40</v>
@@ -6901,7 +7270,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>2041</v>
+        <v>2164</v>
       </c>
       <c r="G8" s="0">
         <v>-20.413798181544415</v>
@@ -6934,21 +7303,21 @@
         <v>0</v>
       </c>
       <c r="Q8" s="0">
-        <v>3.7027709099999999</v>
+        <v>3.261518385</v>
       </c>
       <c r="R8" s="0" t="s">
-        <v>2098</v>
+        <v>2221</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>2016</v>
+        <v>2139</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D9" s="0">
         <v>40</v>
@@ -6957,7 +7326,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>2042</v>
+        <v>2165</v>
       </c>
       <c r="G9" s="0">
         <v>-20.375583471841395</v>
@@ -6990,21 +7359,21 @@
         <v>0</v>
       </c>
       <c r="Q9" s="0">
-        <v>3.7190109439999999</v>
+        <v>3.2750282450000001</v>
       </c>
       <c r="R9" s="0" t="s">
-        <v>2099</v>
+        <v>2222</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>2016</v>
+        <v>2139</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D10" s="0">
         <v>40</v>
@@ -7013,54 +7382,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>2043</v>
+        <v>2166</v>
       </c>
       <c r="G10" s="0">
-        <v>-18.517340012020526</v>
+        <v>-21.139714076268699</v>
       </c>
       <c r="H10" s="0">
-        <v>-17.288772127325529</v>
+        <v>-19.611315093851761</v>
       </c>
       <c r="I10" s="0">
-        <v>-16.316433956580671</v>
+        <v>-18.067521529510614</v>
       </c>
       <c r="J10" s="0">
-        <v>11.861319364831111</v>
+        <v>8.7702969089501703</v>
       </c>
       <c r="K10" s="0">
-        <v>13.663482145775729</v>
+        <v>10.457653435638978</v>
       </c>
       <c r="L10" s="0">
-        <v>15.281933382858302</v>
+        <v>12.491768394311656</v>
       </c>
       <c r="M10" s="0">
-        <v>-33.416263203830674</v>
+        <v>-32.634376921075635</v>
       </c>
       <c r="N10" s="0">
-        <v>-31.766904182880786</v>
+        <v>-31.075228598731989</v>
       </c>
       <c r="O10" s="0">
-        <v>-29.918986385923951</v>
+        <v>-28.716779777174153</v>
       </c>
       <c r="P10" s="0">
         <v>0</v>
       </c>
       <c r="Q10" s="0">
-        <v>18.818759140000001</v>
+        <v>296.823741316</v>
       </c>
       <c r="R10" s="0" t="s">
-        <v>2100</v>
+        <v>2223</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>2016</v>
+        <v>2139</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D11" s="0">
         <v>40</v>
@@ -7069,54 +7438,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>2044</v>
+        <v>2167</v>
       </c>
       <c r="G11" s="0">
-        <v>-18.428017931580531</v>
+        <v>-21.091383952002339</v>
       </c>
       <c r="H11" s="0">
-        <v>-17.207626158643468</v>
+        <v>-19.5793314500729</v>
       </c>
       <c r="I11" s="0">
-        <v>-15.050936563656496</v>
+        <v>-17.869046003021971</v>
       </c>
       <c r="J11" s="0">
-        <v>11.983925580537958</v>
+        <v>8.8192327114107414</v>
       </c>
       <c r="K11" s="0">
-        <v>13.791728274505191</v>
+        <v>10.496232146797535</v>
       </c>
       <c r="L11" s="0">
-        <v>17.678815840769389</v>
+        <v>12.780495738268574</v>
       </c>
       <c r="M11" s="0">
-        <v>-33.276949814968887</v>
+        <v>-32.516750682458813</v>
       </c>
       <c r="N11" s="0">
-        <v>-31.627521812671326</v>
+        <v>-31.010610150909827</v>
       </c>
       <c r="O11" s="0">
-        <v>-29.584606292353975</v>
+        <v>-28.460833681004974</v>
       </c>
       <c r="P11" s="0">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q11" s="0">
-        <v>21.356351737000001</v>
+        <v>300.87647246900002</v>
       </c>
       <c r="R11" s="0" t="s">
-        <v>2101</v>
+        <v>2224</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>2017</v>
+        <v>2140</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D12" s="0">
         <v>40</v>
@@ -7125,7 +7494,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>2045</v>
+        <v>2168</v>
       </c>
       <c r="G12" s="0">
         <v>-5.5798344850129187</v>
@@ -7158,21 +7527,21 @@
         <v>0</v>
       </c>
       <c r="Q12" s="0">
-        <v>3.2278905999999998</v>
+        <v>3.13458053</v>
       </c>
       <c r="R12" s="0" t="s">
-        <v>2102</v>
+        <v>2225</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>2017</v>
+        <v>2140</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D13" s="0">
         <v>40</v>
@@ -7181,7 +7550,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>2046</v>
+        <v>2169</v>
       </c>
       <c r="G13" s="0">
         <v>-21.213114059865443</v>
@@ -7214,21 +7583,21 @@
         <v>0</v>
       </c>
       <c r="Q13" s="0">
-        <v>3.2674530169999998</v>
+        <v>3.1670797149999999</v>
       </c>
       <c r="R13" s="0" t="s">
-        <v>2103</v>
+        <v>2226</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>2017</v>
+        <v>2140</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D14" s="0">
         <v>40</v>
@@ -7237,7 +7606,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>2047</v>
+        <v>2170</v>
       </c>
       <c r="G14" s="0">
         <v>-21.161779043338118</v>
@@ -7270,21 +7639,21 @@
         <v>0</v>
       </c>
       <c r="Q14" s="0">
-        <v>3.2801903559999999</v>
+        <v>3.1787468350000001</v>
       </c>
       <c r="R14" s="0" t="s">
-        <v>2104</v>
+        <v>2227</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>2017</v>
+        <v>2140</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D15" s="0">
         <v>40</v>
@@ -7293,54 +7662,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>2048</v>
+        <v>2171</v>
       </c>
       <c r="G15" s="0">
-        <v>-18.962492219096983</v>
+        <v>-21.558838442819713</v>
       </c>
       <c r="H15" s="0">
-        <v>-12.382231894451985</v>
+        <v>-13.0043952746909</v>
       </c>
       <c r="I15" s="0">
-        <v>-15.345113471650894</v>
+        <v>-16.723700686318171</v>
       </c>
       <c r="J15" s="0">
-        <v>11.268740788174608</v>
+        <v>8.3571477023684224</v>
       </c>
       <c r="K15" s="0">
-        <v>24.037450630995853</v>
+        <v>22.375885769539693</v>
       </c>
       <c r="L15" s="0">
-        <v>17.090089079367473</v>
+        <v>14.5819285425908</v>
       </c>
       <c r="M15" s="0">
-        <v>-33.596101862491295</v>
+        <v>-32.818440655441961</v>
       </c>
       <c r="N15" s="0">
-        <v>-29.292777779182863</v>
+        <v>-27.914199240796556</v>
       </c>
       <c r="O15" s="0">
-        <v>-29.00200151214915</v>
+        <v>-27.396847573490511</v>
       </c>
       <c r="P15" s="0">
         <v>0</v>
       </c>
       <c r="Q15" s="0">
-        <v>14.756190565000001</v>
+        <v>296.74290922500001</v>
       </c>
       <c r="R15" s="0" t="s">
-        <v>2105</v>
+        <v>2228</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>2017</v>
+        <v>2140</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D16" s="0">
         <v>40</v>
@@ -7349,54 +7718,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>2049</v>
+        <v>2172</v>
       </c>
       <c r="G16" s="0">
-        <v>-18.870557836214445</v>
+        <v>-21.503893193431654</v>
       </c>
       <c r="H16" s="0">
-        <v>-12.535996244730704</v>
+        <v>-12.99741284394077</v>
       </c>
       <c r="I16" s="0">
-        <v>-13.377630384625483</v>
+        <v>-16.681165817253998</v>
       </c>
       <c r="J16" s="0">
-        <v>11.388646379185753</v>
+        <v>8.410180956356335</v>
       </c>
       <c r="K16" s="0">
-        <v>23.615665449203764</v>
+        <v>22.393880574297011</v>
       </c>
       <c r="L16" s="0">
-        <v>21.434752872529788</v>
+        <v>14.653511488063886</v>
       </c>
       <c r="M16" s="0">
-        <v>-33.453707844069712</v>
+        <v>-32.69765719837477</v>
       </c>
       <c r="N16" s="0">
-        <v>-29.450232871416869</v>
+        <v>-27.885094141194074</v>
       </c>
       <c r="O16" s="0">
-        <v>-29.694508841357759</v>
+        <v>-27.320057794970086</v>
       </c>
       <c r="P16" s="0">
         <v>6</v>
       </c>
       <c r="Q16" s="0">
-        <v>20.524663129</v>
+        <v>307.38641275100002</v>
       </c>
       <c r="R16" s="0" t="s">
-        <v>2106</v>
+        <v>2229</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>2018</v>
+        <v>2141</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D17" s="0">
         <v>40</v>
@@ -7405,7 +7774,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>2050</v>
+        <v>2173</v>
       </c>
       <c r="G17" s="0">
         <v>-5.4243076236990948</v>
@@ -7438,21 +7807,21 @@
         <v>0</v>
       </c>
       <c r="Q17" s="0">
-        <v>3.2798628540000001</v>
+        <v>3.1959156530000001</v>
       </c>
       <c r="R17" s="0" t="s">
-        <v>2107</v>
+        <v>2230</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>2018</v>
+        <v>2141</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D18" s="0">
         <v>40</v>
@@ -7461,7 +7830,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>2051</v>
+        <v>2174</v>
       </c>
       <c r="G18" s="0">
         <v>-16.657821199109176</v>
@@ -7494,21 +7863,21 @@
         <v>0</v>
       </c>
       <c r="Q18" s="0">
-        <v>3.3177027570000002</v>
+        <v>3.2344585189999999</v>
       </c>
       <c r="R18" s="0" t="s">
-        <v>2108</v>
+        <v>2231</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>2018</v>
+        <v>2141</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D19" s="0">
         <v>40</v>
@@ -7517,7 +7886,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>2052</v>
+        <v>2175</v>
       </c>
       <c r="G19" s="0">
         <v>-16.623145541942378</v>
@@ -7550,21 +7919,21 @@
         <v>0</v>
       </c>
       <c r="Q19" s="0">
-        <v>3.3318787310000002</v>
+        <v>3.2475191730000001</v>
       </c>
       <c r="R19" s="0" t="s">
-        <v>2109</v>
+        <v>2232</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
-        <v>2018</v>
+        <v>2141</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D20" s="0">
         <v>40</v>
@@ -7573,54 +7942,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>2053</v>
+        <v>2176</v>
       </c>
       <c r="G20" s="0">
-        <v>-15.765510411308547</v>
+        <v>-16.970014030536721</v>
       </c>
       <c r="H20" s="0">
-        <v>-15.413412289353687</v>
+        <v>-16.203866387694021</v>
       </c>
       <c r="I20" s="0">
-        <v>-15.712833175948173</v>
+        <v>-16.877994535713441</v>
       </c>
       <c r="J20" s="0">
-        <v>16.282627194886281</v>
+        <v>14.174224218427524</v>
       </c>
       <c r="K20" s="0">
-        <v>16.956233384258887</v>
+        <v>15.481273408813035</v>
       </c>
       <c r="L20" s="0">
-        <v>16.381676342592367</v>
+        <v>14.325186118898374</v>
       </c>
       <c r="M20" s="0">
-        <v>-34.266321357150318</v>
+        <v>-33.50008985554755</v>
       </c>
       <c r="N20" s="0">
-        <v>-32.048412720272054</v>
+        <v>-31.541243418137462</v>
       </c>
       <c r="O20" s="0">
-        <v>-33.199159378304415</v>
+        <v>-32.945708223618468</v>
       </c>
       <c r="P20" s="0">
         <v>0</v>
       </c>
       <c r="Q20" s="0">
-        <v>14.529185151</v>
+        <v>308.89261845300001</v>
       </c>
       <c r="R20" s="0" t="s">
-        <v>2110</v>
+        <v>2233</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
-        <v>2018</v>
+        <v>2141</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D21" s="0">
         <v>40</v>
@@ -7629,54 +7998,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>2054</v>
+        <v>2177</v>
       </c>
       <c r="G21" s="0">
-        <v>-15.724709185970298</v>
+        <v>-16.95193989984293</v>
       </c>
       <c r="H21" s="0">
-        <v>-15.479785634588346</v>
+        <v>-16.192663052050527</v>
       </c>
       <c r="I21" s="0">
-        <v>-15.185472723484644</v>
+        <v>-16.830857590343598</v>
       </c>
       <c r="J21" s="0">
-        <v>16.359293372045162</v>
+        <v>14.203749519949392</v>
       </c>
       <c r="K21" s="0">
-        <v>16.827155895245372</v>
+        <v>15.50125452910776</v>
       </c>
       <c r="L21" s="0">
-        <v>17.407097577985759</v>
+        <v>14.403137956622281</v>
       </c>
       <c r="M21" s="0">
-        <v>-34.036129065753855</v>
+        <v>-33.323305524379116</v>
       </c>
       <c r="N21" s="0">
-        <v>-31.938230202731226</v>
+        <v>-31.465034939243864</v>
       </c>
       <c r="O21" s="0">
-        <v>-33.055650308217757</v>
+        <v>-32.741676169288631</v>
       </c>
       <c r="P21" s="0">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="0">
-        <v>19.209040718000001</v>
+        <v>309.80283089099999</v>
       </c>
       <c r="R21" s="0" t="s">
-        <v>2111</v>
+        <v>2234</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>2019</v>
+        <v>2142</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D22" s="0">
         <v>40</v>
@@ -7685,7 +8054,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>2055</v>
+        <v>2178</v>
       </c>
       <c r="G22" s="0">
         <v>-5.1213170194981199</v>
@@ -7718,21 +8087,21 @@
         <v>0</v>
       </c>
       <c r="Q22" s="0">
-        <v>3.0346654540000002</v>
+        <v>3.2477884509999999</v>
       </c>
       <c r="R22" s="0" t="s">
-        <v>2112</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>2019</v>
+        <v>2142</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D23" s="0">
         <v>40</v>
@@ -7741,7 +8110,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>2056</v>
+        <v>2179</v>
       </c>
       <c r="G23" s="0">
         <v>-20.879145492539042</v>
@@ -7774,21 +8143,21 @@
         <v>0</v>
       </c>
       <c r="Q23" s="0">
-        <v>3.0632812089999999</v>
+        <v>3.288382124</v>
       </c>
       <c r="R23" s="0" t="s">
-        <v>2113</v>
+        <v>2236</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="s">
-        <v>2019</v>
+        <v>2142</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D24" s="0">
         <v>40</v>
@@ -7797,7 +8166,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>2057</v>
+        <v>2180</v>
       </c>
       <c r="G24" s="0">
         <v>-20.827876457576863</v>
@@ -7830,21 +8199,21 @@
         <v>0</v>
       </c>
       <c r="Q24" s="0">
-        <v>3.075331898</v>
+        <v>3.2997039990000001</v>
       </c>
       <c r="R24" s="0" t="s">
-        <v>2114</v>
+        <v>2237</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>2019</v>
+        <v>2142</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D25" s="0">
         <v>40</v>
@@ -7853,54 +8222,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>2058</v>
+        <v>2181</v>
       </c>
       <c r="G25" s="0">
-        <v>-18.767746881301573</v>
+        <v>-21.291244415039429</v>
       </c>
       <c r="H25" s="0">
-        <v>-17.859141726175764</v>
+        <v>-19.972993875707921</v>
       </c>
       <c r="I25" s="0">
-        <v>-17.247947075460889</v>
+        <v>-18.827341275878251</v>
       </c>
       <c r="J25" s="0">
-        <v>11.524249599489599</v>
+        <v>8.6186209210548128</v>
       </c>
       <c r="K25" s="0">
-        <v>12.795077291736233</v>
+        <v>10.031140335207517</v>
       </c>
       <c r="L25" s="0">
-        <v>13.727853827878107</v>
+        <v>11.445451679612919</v>
       </c>
       <c r="M25" s="0">
-        <v>-33.360812205615879</v>
+        <v>-32.581623445491367</v>
       </c>
       <c r="N25" s="0">
-        <v>-31.723920326912094</v>
+        <v>-31.084577371727647</v>
       </c>
       <c r="O25" s="0">
-        <v>-30.061110794227378</v>
+        <v>-29.045288896501535</v>
       </c>
       <c r="P25" s="0">
         <v>0</v>
       </c>
       <c r="Q25" s="0">
-        <v>13.488842471</v>
+        <v>288.041508749</v>
       </c>
       <c r="R25" s="0" t="s">
-        <v>2115</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
-        <v>2019</v>
+        <v>2142</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D26" s="0">
         <v>40</v>
@@ -7909,54 +8278,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>2059</v>
+        <v>2182</v>
       </c>
       <c r="G26" s="0">
-        <v>-18.675733105774594</v>
+        <v>-21.24062169463107</v>
       </c>
       <c r="H26" s="0">
-        <v>-17.770399831718809</v>
+        <v>-19.93846944757582</v>
       </c>
       <c r="I26" s="0">
-        <v>-15.996402098809989</v>
+        <v>-18.656477630915184</v>
       </c>
       <c r="J26" s="0">
-        <v>11.646980402343095</v>
+        <v>8.6689982497500289</v>
       </c>
       <c r="K26" s="0">
-        <v>12.926471958777849</v>
+        <v>10.071091172841518</v>
       </c>
       <c r="L26" s="0">
-        <v>15.855498287431219</v>
+        <v>11.672828866686917</v>
       </c>
       <c r="M26" s="0">
-        <v>-33.222510142135093</v>
+        <v>-32.46597112088692</v>
       </c>
       <c r="N26" s="0">
-        <v>-31.587910415406601</v>
+        <v>-31.021782832366959</v>
       </c>
       <c r="O26" s="0">
-        <v>-29.621764771376682</v>
+        <v>-28.779229466121002</v>
       </c>
       <c r="P26" s="0">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q26" s="0">
-        <v>15.996666600999999</v>
+        <v>291.67890848000002</v>
       </c>
       <c r="R26" s="0" t="s">
-        <v>2116</v>
+        <v>2239</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="s">
-        <v>2020</v>
+        <v>2143</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D27" s="0">
         <v>40</v>
@@ -7965,7 +8334,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>2060</v>
+        <v>2183</v>
       </c>
       <c r="G27" s="0">
         <v>-4.7534033063092922</v>
@@ -7998,21 +8367,21 @@
         <v>0</v>
       </c>
       <c r="Q27" s="0">
-        <v>3.2443867169999998</v>
+        <v>3.1103723150000002</v>
       </c>
       <c r="R27" s="0" t="s">
-        <v>2117</v>
+        <v>2240</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="s">
-        <v>2020</v>
+        <v>2143</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D28" s="0">
         <v>40</v>
@@ -8021,7 +8390,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>2061</v>
+        <v>2184</v>
       </c>
       <c r="G28" s="0">
         <v>-11.354386510528677</v>
@@ -8054,21 +8423,21 @@
         <v>0</v>
       </c>
       <c r="Q28" s="0">
-        <v>3.2747379350000001</v>
+        <v>3.1445157300000002</v>
       </c>
       <c r="R28" s="0" t="s">
-        <v>2118</v>
+        <v>2241</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>2020</v>
+        <v>2143</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D29" s="0">
         <v>40</v>
@@ -8077,7 +8446,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>2062</v>
+        <v>2185</v>
       </c>
       <c r="G29" s="0">
         <v>-11.349889698383695</v>
@@ -8110,21 +8479,21 @@
         <v>0</v>
       </c>
       <c r="Q29" s="0">
-        <v>3.286213735</v>
+        <v>3.1565575909999999</v>
       </c>
       <c r="R29" s="0" t="s">
-        <v>2119</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
-        <v>2020</v>
+        <v>2143</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D30" s="0">
         <v>40</v>
@@ -8133,54 +8502,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>2063</v>
+        <v>2186</v>
       </c>
       <c r="G30" s="0">
-        <v>-11.110585894570637</v>
+        <v>-11.323963795080216</v>
       </c>
       <c r="H30" s="0">
-        <v>-11.067443045227039</v>
+        <v>-11.382438290440227</v>
       </c>
       <c r="I30" s="0">
-        <v>-11.064342442657429</v>
+        <v>-11.373642503722525</v>
       </c>
       <c r="J30" s="0">
-        <v>27.827276625085894</v>
+        <v>27.151999079232841</v>
       </c>
       <c r="K30" s="0">
-        <v>27.965838656065351</v>
+        <v>26.96982233198397</v>
       </c>
       <c r="L30" s="0">
-        <v>27.975823405269029</v>
+        <v>26.997147219427312</v>
       </c>
       <c r="M30" s="0">
-        <v>-33.349939418359</v>
+        <v>-32.555296987550534</v>
       </c>
       <c r="N30" s="0">
-        <v>-32.329379076256195</v>
+        <v>-31.765025910492458</v>
       </c>
       <c r="O30" s="0">
-        <v>-32.480063618854629</v>
+        <v>-32.175749658305726</v>
       </c>
       <c r="P30" s="0">
         <v>0</v>
       </c>
       <c r="Q30" s="0">
-        <v>13.887328258</v>
+        <v>293.47288244100002</v>
       </c>
       <c r="R30" s="0" t="s">
-        <v>2120</v>
+        <v>2243</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="s">
-        <v>2020</v>
+        <v>2143</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D31" s="0">
         <v>40</v>
@@ -8189,54 +8558,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>2064</v>
+        <v>2187</v>
       </c>
       <c r="G31" s="0">
-        <v>-11.098062069106568</v>
+        <v>-11.31916192436152</v>
       </c>
       <c r="H31" s="0">
-        <v>-11.095604560111152</v>
+        <v>-11.378452573110426</v>
       </c>
       <c r="I31" s="0">
-        <v>-10.977867399509034</v>
+        <v>-11.362184374025473</v>
       </c>
       <c r="J31" s="0">
-        <v>27.867428565491725</v>
+        <v>27.167013826240044</v>
       </c>
       <c r="K31" s="0">
-        <v>27.875314245409452</v>
+        <v>26.982200886116324</v>
       </c>
       <c r="L31" s="0">
-        <v>28.255736378903961</v>
+        <v>27.032784436825871</v>
       </c>
       <c r="M31" s="0">
-        <v>-33.206010816273391</v>
+        <v>-32.445135591355012</v>
       </c>
       <c r="N31" s="0">
-        <v>-32.237163397163535</v>
+        <v>-31.692612412685747</v>
       </c>
       <c r="O31" s="0">
-        <v>-32.298380096105326</v>
+        <v>-31.991224733133485</v>
       </c>
       <c r="P31" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q31" s="0">
-        <v>16.780756691000001</v>
+        <v>294.47399337000002</v>
       </c>
       <c r="R31" s="0" t="s">
-        <v>2121</v>
+        <v>2244</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="s">
-        <v>2021</v>
+        <v>2144</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D32" s="0">
         <v>40</v>
@@ -8245,7 +8614,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F32" s="0" t="s">
-        <v>2065</v>
+        <v>2188</v>
       </c>
       <c r="G32" s="0">
         <v>-5.1631376314694233</v>
@@ -8278,21 +8647,21 @@
         <v>0</v>
       </c>
       <c r="Q32" s="0">
-        <v>3.202465868</v>
+        <v>3.2343927350000001</v>
       </c>
       <c r="R32" s="0" t="s">
-        <v>2122</v>
+        <v>2245</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="s">
-        <v>2021</v>
+        <v>2144</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D33" s="0">
         <v>40</v>
@@ -8301,7 +8670,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>2066</v>
+        <v>2189</v>
       </c>
       <c r="G33" s="0">
         <v>-14.170623821597673</v>
@@ -8334,21 +8703,21 @@
         <v>0</v>
       </c>
       <c r="Q33" s="0">
-        <v>3.2326205350000001</v>
+        <v>3.272971144</v>
       </c>
       <c r="R33" s="0" t="s">
-        <v>2123</v>
+        <v>2246</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="s">
-        <v>2021</v>
+        <v>2144</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D34" s="0">
         <v>40</v>
@@ -8357,7 +8726,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>2067</v>
+        <v>2190</v>
       </c>
       <c r="G34" s="0">
         <v>-14.142635028596175</v>
@@ -8390,21 +8759,21 @@
         <v>0</v>
       </c>
       <c r="Q34" s="0">
-        <v>3.243564111</v>
+        <v>3.2843279139999999</v>
       </c>
       <c r="R34" s="0" t="s">
-        <v>2124</v>
+        <v>2247</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="s">
-        <v>2021</v>
+        <v>2144</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D35" s="0">
         <v>40</v>
@@ -8413,54 +8782,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>2068</v>
+        <v>2191</v>
       </c>
       <c r="G35" s="0">
-        <v>-13.593879143194382</v>
+        <v>-13.878642890002817</v>
       </c>
       <c r="H35" s="0">
-        <v>-13.713052491049112</v>
+        <v>-14.63236535796389</v>
       </c>
       <c r="I35" s="0">
-        <v>-12.498232289014544</v>
+        <v>-12.73532452878467</v>
       </c>
       <c r="J35" s="0">
-        <v>20.907689551608751</v>
+        <v>20.233352860843013</v>
       </c>
       <c r="K35" s="0">
-        <v>20.622787912085006</v>
+        <v>18.551615395245996</v>
       </c>
       <c r="L35" s="0">
-        <v>23.718563654825687</v>
+        <v>23.07989206956681</v>
       </c>
       <c r="M35" s="0">
-        <v>-33.126030627426708</v>
+        <v>-32.364781870407036</v>
       </c>
       <c r="N35" s="0">
-        <v>-32.671134288105272</v>
+        <v>-31.778770941616749</v>
       </c>
       <c r="O35" s="0">
-        <v>-28.00483786162502</v>
+        <v>-26.576804197944259</v>
       </c>
       <c r="P35" s="0">
         <v>0</v>
       </c>
       <c r="Q35" s="0">
-        <v>13.760141317</v>
+        <v>302.756353655</v>
       </c>
       <c r="R35" s="0" t="s">
-        <v>2125</v>
+        <v>2248</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0" t="s">
-        <v>2021</v>
+        <v>2144</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>2025</v>
+        <v>2148</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>2029</v>
+        <v>2152</v>
       </c>
       <c r="D36" s="0">
         <v>40</v>
@@ -8469,54 +8838,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>2069</v>
+        <v>2192</v>
       </c>
       <c r="G36" s="0">
-        <v>-13.57383621758925</v>
+        <v>-13.868353791263623</v>
       </c>
       <c r="H36" s="0">
-        <v>-13.708595750455032</v>
+        <v>-14.623742217371047</v>
       </c>
       <c r="I36" s="0">
-        <v>-11.615093380930411</v>
+        <v>-12.673837511166042</v>
       </c>
       <c r="J36" s="0">
-        <v>20.955990317783989</v>
+        <v>20.257335012020675</v>
       </c>
       <c r="K36" s="0">
-        <v>20.633372204954082</v>
+        <v>18.5700421344152</v>
       </c>
       <c r="L36" s="0">
-        <v>26.257013711404227</v>
+        <v>23.243853227695531</v>
       </c>
       <c r="M36" s="0">
-        <v>-32.948340155685457</v>
+        <v>-32.236947820458589</v>
       </c>
       <c r="N36" s="0">
-        <v>-32.676012312591396</v>
+        <v>-31.693603865722562</v>
       </c>
       <c r="O36" s="0">
-        <v>-28.452441521775004</v>
+        <v>-26.35438783544388</v>
       </c>
       <c r="P36" s="0">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="Q36" s="0">
-        <v>19.229824382</v>
+        <v>308.88823636699999</v>
       </c>
       <c r="R36" s="0" t="s">
-        <v>2126</v>
+        <v>2249</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="s">
-        <v>2022</v>
+        <v>2145</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>2026</v>
+        <v>2149</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>2030</v>
+        <v>2153</v>
       </c>
       <c r="D37" s="0">
         <v>50</v>
@@ -8525,7 +8894,7 @@
         <v>2.9225607135647587</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>2070</v>
+        <v>2193</v>
       </c>
       <c r="G37" s="0">
         <v>-4.1302089576645553</v>
@@ -8558,21 +8927,21 @@
         <v>0</v>
       </c>
       <c r="Q37" s="0">
-        <v>26.862219263</v>
+        <v>17.979999305</v>
       </c>
       <c r="R37" s="0" t="s">
-        <v>2127</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="s">
-        <v>2022</v>
+        <v>2145</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>2026</v>
+        <v>2149</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>2030</v>
+        <v>2153</v>
       </c>
       <c r="D38" s="0">
         <v>50</v>
@@ -8581,7 +8950,7 @@
         <v>2.9225607135647587</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>2071</v>
+        <v>2194</v>
       </c>
       <c r="G38" s="0">
         <v>-13.755479845770818</v>
@@ -8614,21 +8983,21 @@
         <v>0</v>
       </c>
       <c r="Q38" s="0">
-        <v>26.900333181000001</v>
+        <v>18.022543403</v>
       </c>
       <c r="R38" s="0" t="s">
-        <v>2128</v>
+        <v>2251</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="s">
-        <v>2022</v>
+        <v>2145</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>2026</v>
+        <v>2149</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>2030</v>
+        <v>2153</v>
       </c>
       <c r="D39" s="0">
         <v>50</v>
@@ -8637,7 +9006,7 @@
         <v>2.9225607135647587</v>
       </c>
       <c r="F39" s="0" t="s">
-        <v>2072</v>
+        <v>2195</v>
       </c>
       <c r="G39" s="0">
         <v>-13.710503862148455</v>
@@ -8670,21 +9039,21 @@
         <v>0</v>
       </c>
       <c r="Q39" s="0">
-        <v>26.915695311</v>
+        <v>18.037512418999999</v>
       </c>
       <c r="R39" s="0" t="s">
-        <v>2129</v>
+        <v>2252</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="0" t="s">
-        <v>2022</v>
+        <v>2145</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>2026</v>
+        <v>2149</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>2030</v>
+        <v>2153</v>
       </c>
       <c r="D40" s="0">
         <v>50</v>
@@ -8693,54 +9062,54 @@
         <v>2.9225607135647587</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>2073</v>
+        <v>2196</v>
       </c>
       <c r="G40" s="0">
-        <v>-13.263641021981961</v>
+        <v>-13.733683994044693</v>
       </c>
       <c r="H40" s="0">
-        <v>-13.231390509005426</v>
+        <v>-13.824509093439566</v>
       </c>
       <c r="I40" s="0">
-        <v>-11.88885094531769</v>
+        <v>-11.319255828948611</v>
       </c>
       <c r="J40" s="0">
-        <v>21.717905991481544</v>
+        <v>20.573860950069211</v>
       </c>
       <c r="K40" s="0">
-        <v>21.798693977406977</v>
+        <v>20.359848654096144</v>
       </c>
       <c r="L40" s="0">
-        <v>25.442363474087273</v>
+        <v>27.166720120755411</v>
       </c>
       <c r="M40" s="0">
-        <v>-31.776330797674387</v>
+        <v>-30.371983444890876</v>
       </c>
       <c r="N40" s="0">
-        <v>-30.128866091541195</v>
+        <v>-27.352756927378312</v>
       </c>
       <c r="O40" s="0">
-        <v>-27.153203976607898</v>
+        <v>-23.606445269577371</v>
       </c>
       <c r="P40" s="0">
         <v>0</v>
       </c>
       <c r="Q40" s="0">
-        <v>41.093642496999998</v>
+        <v>548.595573737</v>
       </c>
       <c r="R40" s="0" t="s">
-        <v>2130</v>
+        <v>2253</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="0" t="s">
-        <v>2022</v>
+        <v>2145</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>2026</v>
+        <v>2149</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>2030</v>
+        <v>2153</v>
       </c>
       <c r="D41" s="0">
         <v>50</v>
@@ -8749,54 +9118,54 @@
         <v>2.9225607135647587</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>2074</v>
+        <v>2197</v>
       </c>
       <c r="G41" s="0">
-        <v>-13.225410864084131</v>
+        <v>-13.723601380689951</v>
       </c>
       <c r="H41" s="0">
-        <v>-13.210622648538596</v>
+        <v>-13.614963702783101</v>
       </c>
       <c r="I41" s="0">
-        <v>-12.05843562410738</v>
+        <v>-11.175312165483762</v>
       </c>
       <c r="J41" s="0">
-        <v>21.813706064077458</v>
+        <v>20.597757031874625</v>
       </c>
       <c r="K41" s="0">
-        <v>21.850876758929687</v>
+        <v>20.856998737930962</v>
       </c>
       <c r="L41" s="0">
-        <v>24.95044057462416</v>
+        <v>27.62068161247926</v>
       </c>
       <c r="M41" s="0">
-        <v>-31.568174544009977</v>
+        <v>-30.29225174639415</v>
       </c>
       <c r="N41" s="0">
-        <v>-30.580289384915783</v>
+        <v>-27.078308610095444</v>
       </c>
       <c r="O41" s="0">
-        <v>-28.401568236771553</v>
+        <v>-23.309394524550626</v>
       </c>
       <c r="P41" s="0">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Q41" s="0">
-        <v>47.806039413999997</v>
+        <v>560.37258802500003</v>
       </c>
       <c r="R41" s="0" t="s">
-        <v>2131</v>
+        <v>2254</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="0" t="s">
-        <v>2023</v>
+        <v>2146</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>2027</v>
+        <v>2150</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>2031</v>
+        <v>2154</v>
       </c>
       <c r="D42" s="0">
         <v>40</v>
@@ -8805,7 +9174,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>2075</v>
+        <v>2198</v>
       </c>
       <c r="G42" s="0">
         <v>-5.1631376314694233</v>
@@ -8838,21 +9207,21 @@
         <v>0</v>
       </c>
       <c r="Q42" s="0">
-        <v>3.1344335390000002</v>
+        <v>3.2149822110000001</v>
       </c>
       <c r="R42" s="0" t="s">
-        <v>2132</v>
+        <v>2255</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="0" t="s">
-        <v>2023</v>
+        <v>2146</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>2027</v>
+        <v>2150</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>2031</v>
+        <v>2154</v>
       </c>
       <c r="D43" s="0">
         <v>40</v>
@@ -8861,7 +9230,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F43" s="0" t="s">
-        <v>2076</v>
+        <v>2199</v>
       </c>
       <c r="G43" s="0">
         <v>-14.170623821597673</v>
@@ -8894,21 +9263,21 @@
         <v>0</v>
       </c>
       <c r="Q43" s="0">
-        <v>3.163203051</v>
+        <v>3.2496189919999998</v>
       </c>
       <c r="R43" s="0" t="s">
-        <v>2133</v>
+        <v>2256</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="0" t="s">
-        <v>2023</v>
+        <v>2146</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>2027</v>
+        <v>2150</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>2031</v>
+        <v>2154</v>
       </c>
       <c r="D44" s="0">
         <v>40</v>
@@ -8917,7 +9286,7 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F44" s="0" t="s">
-        <v>2077</v>
+        <v>2200</v>
       </c>
       <c r="G44" s="0">
         <v>-14.142635028596175</v>
@@ -8950,21 +9319,21 @@
         <v>0</v>
       </c>
       <c r="Q44" s="0">
-        <v>3.1749524739999999</v>
+        <v>3.2612535619999998</v>
       </c>
       <c r="R44" s="0" t="s">
-        <v>2134</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="0" t="s">
-        <v>2023</v>
+        <v>2146</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>2027</v>
+        <v>2150</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>2031</v>
+        <v>2154</v>
       </c>
       <c r="D45" s="0">
         <v>40</v>
@@ -8973,54 +9342,54 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F45" s="0" t="s">
-        <v>2078</v>
+        <v>2201</v>
       </c>
       <c r="G45" s="0">
-        <v>-13.593879143194382</v>
+        <v>-13.878642890002817</v>
       </c>
       <c r="H45" s="0">
-        <v>-13.713052491049112</v>
+        <v>-14.63236535796389</v>
       </c>
       <c r="I45" s="0">
-        <v>-12.498232289014544</v>
+        <v>-12.73532452878467</v>
       </c>
       <c r="J45" s="0">
-        <v>20.907689551608751</v>
+        <v>20.233352860843013</v>
       </c>
       <c r="K45" s="0">
-        <v>20.622787912085006</v>
+        <v>18.551615395245996</v>
       </c>
       <c r="L45" s="0">
-        <v>23.718563654825687</v>
+        <v>23.07989206956681</v>
       </c>
       <c r="M45" s="0">
-        <v>-33.126030627426708</v>
+        <v>-32.364781870407036</v>
       </c>
       <c r="N45" s="0">
-        <v>-32.671134288105272</v>
+        <v>-31.778770941616749</v>
       </c>
       <c r="O45" s="0">
-        <v>-28.00483786162502</v>
+        <v>-26.576804197944259</v>
       </c>
       <c r="P45" s="0">
         <v>0</v>
       </c>
       <c r="Q45" s="0">
-        <v>13.499812687</v>
+        <v>297.69969716499998</v>
       </c>
       <c r="R45" s="0" t="s">
-        <v>2135</v>
+        <v>2258</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="0" t="s">
-        <v>2023</v>
+        <v>2146</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>2027</v>
+        <v>2150</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>2031</v>
+        <v>2154</v>
       </c>
       <c r="D46" s="0">
         <v>40</v>
@@ -9029,43 +9398,43 @@
         <v>2.9225607135647595</v>
       </c>
       <c r="F46" s="0" t="s">
-        <v>2079</v>
+        <v>2202</v>
       </c>
       <c r="G46" s="0">
-        <v>-13.458478326130276</v>
+        <v>-13.805327827375448</v>
       </c>
       <c r="H46" s="0">
-        <v>-13.720999410873741</v>
+        <v>-14.670127700036685</v>
       </c>
       <c r="I46" s="0">
-        <v>-11.509975189682365</v>
+        <v>-12.764422341767489</v>
       </c>
       <c r="J46" s="0">
-        <v>21.236164640375616</v>
+        <v>20.404859495118373</v>
       </c>
       <c r="K46" s="0">
-        <v>20.603928278875273</v>
+        <v>18.471136384267155</v>
       </c>
       <c r="L46" s="0">
-        <v>26.57671140897714</v>
+        <v>23.002703574682318</v>
       </c>
       <c r="M46" s="0">
-        <v>-32.9743456510868</v>
+        <v>-32.212961011387293</v>
       </c>
       <c r="N46" s="0">
-        <v>-32.595685806214917</v>
+        <v>-31.751711790011328</v>
       </c>
       <c r="O46" s="0">
-        <v>-27.880060125320789</v>
+        <v>-26.681260731014603</v>
       </c>
       <c r="P46" s="0">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q46" s="0">
-        <v>17.350384359</v>
+        <v>305.30603315299999</v>
       </c>
       <c r="R46" s="0" t="s">
-        <v>2136</v>
+        <v>2259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>